<commit_message>
🔄 Atualização automática - 11/09/2026 23:56:33 (Horário de Brasília)
</commit_message>
<xml_diff>
--- a/dados/indicadores_sao_leopoldo.xlsx
+++ b/dados/indicadores_sao_leopoldo.xlsx
@@ -536,16 +536,16 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
-        <v>338</v>
+        <v>386</v>
       </c>
       <c r="E6" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F6" t="n">
-        <v>171</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🔄 Atualização automática - 09/10/2026 01:22:48 (Horário de Brasília)
</commit_message>
<xml_diff>
--- a/dados/indicadores_sao_leopoldo.xlsx
+++ b/dados/indicadores_sao_leopoldo.xlsx
@@ -453,19 +453,19 @@
         <v>2022</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>603</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>420</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -473,19 +473,19 @@
         <v>2023</v>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>571</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>417</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -493,19 +493,19 @@
         <v>2024</v>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>553</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>380</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -513,19 +513,19 @@
         <v>2025</v>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>651</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>344</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -536,16 +536,16 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>386</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>187</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>